<commit_message>
docs: refresh Chinese delivery summaries
</commit_message>
<xml_diff>
--- a/bug_summary.xlsx
+++ b/bug_summary.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>When multiple sensors report traffic for the same intersection at the same time, aggregate the readings without losing vehicle volume or corrupting the average speed.</t>
+          <t>修复并发交通流量聚合导致路口流量快照损坏的问题。</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Find why querying an offline device without a heartbeat record can crash the device status endpoint, and identify the safe behavior.</t>
+          <t>设备没有心跳记录时，安排下一次巡检不得发生空指针崩溃。</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Make repeated reachable-road queries return independent paths without one query changing the result of another query.</t>
+          <t>路网可达性分析返回结果后，不得继续污染原始道路列表。</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Find why a timing-plan approval failure loses its business error code and explain how the handler should preserve it.</t>
+          <t>配时方案审核失败时必须返回错误，不能静默接受无效审核。</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Stop a cancelled simulation promptly and prevent cancelled work from writing a completed result.</t>
+          <t>仿真请求被取消后，正在运行的仿真任务必须及时停止。</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Ensure concurrent congestion threshold evaluations create only one active event for the same intersection and condition.</t>
+          <t>多个网关同时上报时，批量更新设备状态必须保证并发安全。</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Find why optimization recommendation can dereference a missing baseline plan and define the expected empty-result behavior.</t>
+          <t>没有巡检记录时，维护状态计算不能索引空切片。</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Copy signal phases deeply so changing movements in a copied phase does not mutate the original timing plan.</t>
+          <t>复制信号配置后，相位放行方向必须与原方案相互独立。</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Find why a failed CSV writer can still produce a successful export response and identify the missing error propagation.</t>
+          <t>交通 CSV 导出写入失败时，接口必须返回明确错误。</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Release a dashboard subscriber when its HTTP client disconnects so publishers cannot block on a dead stream.</t>
+          <t>客户端断开后，实时 SSE 交通流发送不能永久阻塞。</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Prevent a stale heartbeat from changing a device back to online after an administrator disables it concurrently.</t>
+          <t>过期心跳到达时，已禁用的信号设备不得被错误恢复。</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Find why calculating metrics for an intersection with no traffic samples can access an absent aggregate and define safe zero metrics.</t>
+          <t>路口没有交通样本时，指标计算必须返回安全的空结果。</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Make OD matrix filtering return a new pair slice so filtering a report cannot modify the stored matrix.</t>
+          <t>筛选 OD 矩阵时，不得修改调用方持有的原始观测数据。</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Find why invalid weather observations are silently replaced with default weather and explain how validation errors should surface.</t>
+          <t>天气观测字段非法时，系统必须拒绝数据而不是静默替换默认值。</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Release a timed-out background job and its queue slot when the job context expires.</t>
+          <t>后台交通任务超过截止时间后，必须通过 context 取消执行。</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Find why concurrent corridor offset updates can expose a partially updated plan to readers.</t>
+          <t>干线协调发布 offset 时，并发读取者必须看到完整一致的快照。</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Schedule an inspection safely when the device lookup is missing instead of dereferencing an absent device.</t>
+          <t>设备查询结果为空时，安排巡检必须安全处理而不能解引用 nil。</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Keep event response state consistent when one action fails while a multi-action response plan is being applied.</t>
+          <t>事件响应计划中后续动作失败时，之前已启动的动作必须回滚。</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Find why sorting compliance findings changes a caller-owned slice and explain the required ownership rule.</t>
+          <t>合规结果排序不能改变调用方拥有的 accepted 切片顺序。</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Do not publish an expired forecast result after the request context has been cancelled.</t>
+          <t>交通预测请求过期或取消后，系统不得继续发布预测结果。</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Prevent concurrent adaptive decisions from overwriting a newer timing-plan version.</t>
+          <t>自适应信号并发更新时，较新的配时方案版本不能被旧写入覆盖。</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Find why capacity assessment can access a missing approach configuration and define the expected diagnostic result.</t>
+          <t>容量评估缺少进口道配置时，必须返回可诊断结果而不能发生空指针崩溃。</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Return an explicit error for an unknown vehicle emission factor instead of silently omitting the vehicle.</t>
+          <t>遇到未知车型排放因子时，排放报表必须返回明确错误。</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Find why an expired priority request may still be granted by a delayed decision task.</t>
+          <t>延迟执行的优先控制任务不得授予已经取消的紧急请求。</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Snapshot alert data independently so later zone evaluations cannot mutate historical alert records.</t>
+          <t>地理围栏重复评估时，新告警不得覆盖历史告警记录。</t>
         </is>
       </c>
     </row>

</xml_diff>